<commit_message>
Label Digital Gateway/Compass buildings as Denied; add county_layer_status
</commit_message>
<xml_diff>
--- a/dc-applications-list.xlsx
+++ b/dc-applications-list.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -458,6 +458,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
@@ -583,204 +584,236 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>Denied</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>2</v>
+      </c>
+      <c r="C10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" t="n">
+        <v>10700000</v>
+      </c>
+      <c r="E10" t="n">
+        <v>875.6</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>Void / Withdrawn / Denied</t>
         </is>
       </c>
-      <c r="B10" t="n">
-        <v>10</v>
-      </c>
-      <c r="C10" t="n">
-        <v>3</v>
-      </c>
-      <c r="D10" t="n">
-        <v>22255200</v>
-      </c>
-      <c r="E10" t="n">
-        <v>1759.8</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="1" t="inlineStr">
+      <c r="B11" t="n">
+        <v>8</v>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="n">
+        <v>11555200</v>
+      </c>
+      <c r="E11" t="n">
+        <v>884.2</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B11">
-        <f>SUM(B5:B10)</f>
+      <c r="B12">
+        <f>SUM(B5:B11)</f>
         <v/>
       </c>
-      <c r="C11">
-        <f>SUM(C5:C10)</f>
+      <c r="C12">
+        <f>SUM(C5:C11)</f>
         <v/>
       </c>
-      <c r="D11">
-        <f>SUM(D5:D10)</f>
+      <c r="D12">
+        <f>SUM(D5:D11)</f>
         <v/>
       </c>
-      <c r="E11">
-        <f>SUM(E5:E10)</f>
+      <c r="E12">
+        <f>SUM(E5:E11)</f>
         <v/>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="1" t="inlineStr">
+    <row r="13"/>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
         <is>
           <t>County raw status (campus layer 10)</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>Campuses</t>
         </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>53</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>15</v>
+        <v>53</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="B16" t="n">
+      <c r="B17" t="n">
         <v>10</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="1" t="inlineStr">
-        <is>
-          <t>Buildings (layer 9) by status</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
+    <row r="18"/>
+    <row r="19">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>Buildings (layer 9) by status shown (county label in county_layer_status)</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
         <is>
           <t>Buildings</t>
         </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>91</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>68</v>
+        <v>91</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Completed</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>59</v>
+        <v>31</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>Denied</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>Under Construction</t>
         </is>
       </c>
-      <c r="B22" t="n">
+      <c r="B24" t="n">
         <v>29</v>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="1" t="inlineStr">
+    <row r="25"/>
+    <row r="26">
+      <c r="A26" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>One row per campus (78 in layer 10; some share a case number) plus ePortal-only projects not in the campus layer (10).</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Buildings joined to campuses by spatial point-in-polygon (all 247 fall in exactly one campus); building PlanningCaseNumber disagrees with campus case number for 21 (see Buildings sheet).</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Stage rules: plan section 5. Precedence Under Construction &gt; county campus status. Completed = campus ProjectStatus Completed. Planned -&gt; Approved / Planned. Pending -&gt; Pending / Under Review (sub-state in county_status_pending_case, e.g. Deferred, Suspended).</t>
+          <t>One row per campus (78 in layer 10; some share a case number) plus ePortal-only projects not in the campus layer (10).</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Digital Gateway North/South and Compass (REZ2022-00032/-33/-36) set to Void per instruction; the county pending-case layer still lists them as Suspended (On-Hold).</t>
+          <t>Buildings joined to campuses by spatial point-in-polygon (all 247 fall in exactly one campus); building PlanningCaseNumber disagrees with campus case number for 21 (see Buildings sheet).</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Pending-case layer: 9 'DATA CENTER' description matches included (7 by campus case number; SUP2026-00035 and SUP2027-00008 attached to Southgate South and Gardner Property by project name). Other pending-layer companion cases joined by case number or exact name.</t>
+          <t>Stage rules: plan section 5. Precedence Under Construction &gt; county campus status. Completed = campus ProjectStatus Completed. Planned -&gt; Approved / Planned. Pending -&gt; Pending / Under Review (sub-state in county_status_pending_case, e.g. Deferred, Suspended).</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ePortal 'data center' keyword search (1,094 hits, noisy) joined by case number, then building GPIN, then case number cited in description, then exact/unique-prefix name. Join method is shown per case in eportal_related_cases.</t>
+          <t>Denied (Oct 15, 2026 edit): Digital Gateway North/South (REZ2022-00032/-33) stage set to 'Denied' and Compass (REZ2022-00036) kept as 'Void / Withdrawn / Denied' (no evidence found it was denied). The 37 buildings of all three (12+8+17) show BuildingStatus 'Denied' (per Patrick: Digital Gateway denied; Compass buildings shown with them); the county layer label ('Pending') is kept in Buildings.county_layer_status. The county pending-case layer still lists the three as Suspended (On-Hold).</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ePortal-only rows: stage from ePortal case status; acreage/district filled only if the case is also in the pending-case layer; otherwise blank. Public facility (substation) reviews excluded.</t>
+          <t>Pending-case layer: 9 'DATA CENTER' description matches included (7 by campus case number; SUP2026-00035 and SUP2027-00008 attached to Southgate South and Gardner Property by project name). Other pending-layer companion cases joined by case number or exact name.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Blank = not available in the sources. MW, applicant/owner not in these sources.</t>
+          <t>ePortal 'data center' keyword search (1,094 hits, noisy) joined by case number, then building GPIN, then case number cited in description, then exact/unique-prefix name. Join method is shown per case in eportal_related_cases.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
+        <is>
+          <t>ePortal-only rows: stage from ePortal case status; acreage/district filled only if the case is also in the pending-case layer; otherwise blank. Public facility (substation) reviews excluded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Blank = not available in the sources. MW, applicant/owner not in these sources.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
         <is>
           <t>last_edit_date = latest LastEditDate among campus and its buildings (county GIS edit, not filing date).</t>
         </is>
@@ -10770,7 +10803,7 @@
       </c>
       <c r="K81" t="inlineStr">
         <is>
-          <t>Override: Digital Gateway/Compass REZ voided (plan §5.4; user instruction); county pending-case layer still shows Suspended (On-Hold)</t>
+          <t>Override: Digital Gateway/Compass REZ voided (plan §5.4; user instruction); county pending-case layer still shows Suspended (On-Hold); building status shown as Denied (user: Digital Gateway denied); original county label kept in Buildings.county_layer_status</t>
         </is>
       </c>
       <c r="L81" t="n">
@@ -10787,7 +10820,7 @@
       </c>
       <c r="P81" t="inlineStr">
         <is>
-          <t>Pending: 17</t>
+          <t>Denied: 17</t>
         </is>
       </c>
       <c r="Q81" t="n">
@@ -10810,7 +10843,7 @@
       </c>
       <c r="W81" t="inlineStr">
         <is>
-          <t>Compass Data Centers (Pending); Compass Data Centers (Pending); Compass Data Centers (Pending); Compass Data Centers (Pending); Compass Data Centers (Pending); Compass Data Centers (Pending); Compass Data Centers (Pending); Compass Data Centers (Pending); Compass Data Centers (Pending); Compass Data Centers (Pending); Compass Data Centers (Pending); Compass Data Centers (Pending); Compass Data Centers (Pending); Compass Data Centers (Pending); Compass Data Centers (Pending); Compass Data Centers (Pending); Compass Data Centers (Pending)</t>
+          <t>Compass Data Centers (Denied); Compass Data Centers (Denied); Compass Data Centers (Denied); Compass Data Centers (Denied); Compass Data Centers (Denied); Compass Data Centers (Denied); Compass Data Centers (Denied); Compass Data Centers (Denied); Compass Data Centers (Denied); Compass Data Centers (Denied); Compass Data Centers (Denied); Compass Data Centers (Denied); Compass Data Centers (Denied); Compass Data Centers (Denied); Compass Data Centers (Denied); Compass Data Centers (Denied); Compass Data Centers (Denied)</t>
         </is>
       </c>
       <c r="Y81" t="inlineStr">
@@ -10941,7 +10974,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>Void / Withdrawn / Denied</t>
+          <t>Denied</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
@@ -10956,7 +10989,7 @@
       </c>
       <c r="K83" t="inlineStr">
         <is>
-          <t>Override: Digital Gateway/Compass REZ voided (plan §5.4; user instruction); county pending-case layer still shows Suspended (On-Hold)</t>
+          <t>Override: Digital Gateway/Compass REZ voided (plan §5.4; user instruction); county pending-case layer still shows Suspended (On-Hold); building status shown as Denied (user: Digital Gateway denied); original county label kept in Buildings.county_layer_status</t>
         </is>
       </c>
       <c r="L83" t="n">
@@ -10973,7 +11006,7 @@
       </c>
       <c r="P83" t="inlineStr">
         <is>
-          <t>Pending: 12</t>
+          <t>Denied: 12</t>
         </is>
       </c>
       <c r="Q83" t="n">
@@ -10996,7 +11029,7 @@
       </c>
       <c r="W83" t="inlineStr">
         <is>
-          <t>Digital Gateway North (Pending); Digital Gateway North (Pending); Digital Gateway North (Pending); Digital Gateway North (Pending); Digital Gateway North (Pending); Digital Gateway North (Pending); Digital Gateway North (Pending); Digital Gateway North (Pending); Digital Gateway North (Pending); Digital Gateway North (Pending); Digital Gateway North (Pending); Digital Gateway North (Pending)</t>
+          <t>Digital Gateway North (Denied); Digital Gateway North (Denied); Digital Gateway North (Denied); Digital Gateway North (Denied); Digital Gateway North (Denied); Digital Gateway North (Denied); Digital Gateway North (Denied); Digital Gateway North (Denied); Digital Gateway North (Denied); Digital Gateway North (Denied); Digital Gateway North (Denied); Digital Gateway North (Denied)</t>
         </is>
       </c>
       <c r="Y83" t="inlineStr">
@@ -11054,7 +11087,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>Void / Withdrawn / Denied</t>
+          <t>Denied</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
@@ -11069,7 +11102,7 @@
       </c>
       <c r="K84" t="inlineStr">
         <is>
-          <t>Override: Digital Gateway/Compass REZ voided (plan §5.4; user instruction); county pending-case layer still shows Suspended (On-Hold)</t>
+          <t>Override: Digital Gateway/Compass REZ voided (plan §5.4; user instruction); county pending-case layer still shows Suspended (On-Hold); building status shown as Denied (user: Digital Gateway denied); original county label kept in Buildings.county_layer_status</t>
         </is>
       </c>
       <c r="L84" t="n">
@@ -11086,7 +11119,7 @@
       </c>
       <c r="P84" t="inlineStr">
         <is>
-          <t>Pending: 8</t>
+          <t>Denied: 8</t>
         </is>
       </c>
       <c r="Q84" t="n">
@@ -11109,7 +11142,7 @@
       </c>
       <c r="W84" t="inlineStr">
         <is>
-          <t>Digital Gateway South (Pending); Digital Gateway South (Pending); Digital Gateway South (Pending); Digital Gateway South (Pending); Digital Gateway South (Pending); Digital Gateway South (Pending); Digital Gateway South (Pending); Digital Gateway South (Pending)</t>
+          <t>Digital Gateway South (Denied); Digital Gateway South (Denied); Digital Gateway South (Denied); Digital Gateway South (Denied); Digital Gateway South (Denied); Digital Gateway South (Denied); Digital Gateway South (Denied); Digital Gateway South (Denied)</t>
         </is>
       </c>
       <c r="Y84" t="inlineStr">
@@ -11515,10 +11548,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P248"/>
+  <dimension ref="A1:Q248"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -11602,6 +11636,11 @@
           <t>source_url</t>
         </is>
       </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>county_layer_status</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -11663,6 +11702,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/242?f=html</t>
         </is>
       </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -11724,6 +11768,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/234?f=html</t>
         </is>
       </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -11780,6 +11829,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/75?f=html</t>
         </is>
       </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -11849,6 +11903,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/14?f=html</t>
         </is>
       </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -11918,6 +11977,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/15?f=html</t>
         </is>
       </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -11987,6 +12051,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/16?f=html</t>
         </is>
       </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -12056,6 +12125,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/13?f=html</t>
         </is>
       </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -12117,6 +12191,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/134?f=html</t>
         </is>
       </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -12178,6 +12257,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/132?f=html</t>
         </is>
       </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -12247,6 +12331,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/27?f=html</t>
         </is>
       </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -12316,6 +12405,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/28?f=html</t>
         </is>
       </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -12390,6 +12484,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/20?f=html</t>
         </is>
       </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -12464,6 +12563,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/19?f=html</t>
         </is>
       </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -12538,6 +12642,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/18?f=html</t>
         </is>
       </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -12612,6 +12721,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/17?f=html</t>
         </is>
       </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -12673,6 +12787,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/233?f=html</t>
         </is>
       </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -12742,6 +12861,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/69?f=html</t>
         </is>
       </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -12811,6 +12935,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/70?f=html</t>
         </is>
       </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -12880,6 +13009,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/67?f=html</t>
         </is>
       </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -12949,6 +13083,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/106?f=html</t>
         </is>
       </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -13018,6 +13157,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/105?f=html</t>
         </is>
       </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -13087,6 +13231,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/107?f=html</t>
         </is>
       </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -13156,6 +13305,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/109?f=html</t>
         </is>
       </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -13225,6 +13379,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/108?f=html</t>
         </is>
       </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -13286,6 +13445,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/136?f=html</t>
         </is>
       </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -13347,6 +13511,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/137?f=html</t>
         </is>
       </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -13408,6 +13577,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/135?f=html</t>
         </is>
       </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -13469,6 +13643,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/138?f=html</t>
         </is>
       </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -13530,6 +13709,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/139?f=html</t>
         </is>
       </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -13591,6 +13775,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/244?f=html</t>
         </is>
       </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -13665,6 +13854,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/46?f=html</t>
         </is>
       </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -13739,6 +13933,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/48?f=html</t>
         </is>
       </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -13813,6 +14012,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/49?f=html</t>
         </is>
       </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -13887,6 +14091,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/47?f=html</t>
         </is>
       </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -13956,6 +14165,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/35?f=html</t>
         </is>
       </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -14025,6 +14239,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/36?f=html</t>
         </is>
       </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -14086,6 +14305,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/100?f=html</t>
         </is>
       </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>Under Construction</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -14147,6 +14371,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/99?f=html</t>
         </is>
       </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>Under Construction</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -14208,6 +14437,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/98?f=html</t>
         </is>
       </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>Under Construction</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -14269,6 +14503,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/97?f=html</t>
         </is>
       </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>Under Construction</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -14338,6 +14577,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/10?f=html</t>
         </is>
       </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -14407,6 +14651,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/9?f=html</t>
         </is>
       </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -14468,6 +14717,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/141?f=html</t>
         </is>
       </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -14529,6 +14783,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/162?f=html</t>
         </is>
       </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -14590,6 +14849,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/251?f=html</t>
         </is>
       </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -14651,6 +14915,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/252?f=html</t>
         </is>
       </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -14712,6 +14981,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/255?f=html</t>
         </is>
       </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -14773,6 +15047,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/254?f=html</t>
         </is>
       </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -14834,6 +15113,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/253?f=html</t>
         </is>
       </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -14895,6 +15179,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/682?f=html</t>
         </is>
       </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -14956,6 +15245,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/260?f=html</t>
         </is>
       </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -15017,6 +15311,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/259?f=html</t>
         </is>
       </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -15086,6 +15385,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/51?f=html</t>
         </is>
       </c>
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -15155,6 +15459,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/50?f=html</t>
         </is>
       </c>
+      <c r="Q55" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -15214,6 +15523,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/53?f=html</t>
         </is>
       </c>
+      <c r="Q56" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -15273,6 +15587,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/54?f=html</t>
         </is>
       </c>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -15332,6 +15651,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/55?f=html</t>
         </is>
       </c>
+      <c r="Q58" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -15393,6 +15717,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/52?f=html</t>
         </is>
       </c>
+      <c r="Q59" t="inlineStr">
+        <is>
+          <t>Under Construction</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -15452,6 +15781,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/130?f=html</t>
         </is>
       </c>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -15511,6 +15845,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/131?f=html</t>
         </is>
       </c>
+      <c r="Q61" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -15577,6 +15916,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/56?f=html</t>
         </is>
       </c>
+      <c r="Q62" t="inlineStr">
+        <is>
+          <t>Under Construction</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -15638,6 +15982,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/205?f=html</t>
         </is>
       </c>
+      <c r="Q63" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -15704,6 +16053,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/62?f=html</t>
         </is>
       </c>
+      <c r="Q64" t="inlineStr">
+        <is>
+          <t>Under Construction</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -15770,6 +16124,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/61?f=html</t>
         </is>
       </c>
+      <c r="Q65" t="inlineStr">
+        <is>
+          <t>Under Construction</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -15836,6 +16195,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/265?f=html</t>
         </is>
       </c>
+      <c r="Q66" t="inlineStr">
+        <is>
+          <t>Under Construction</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -15910,6 +16274,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/34?f=html</t>
         </is>
       </c>
+      <c r="Q67" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -15922,7 +16291,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Denied</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -15959,6 +16328,11 @@
       <c r="P68" t="inlineStr">
         <is>
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/297?f=html</t>
+        </is>
+      </c>
+      <c r="Q68" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
     </row>
@@ -15973,7 +16347,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Denied</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -16010,6 +16384,11 @@
       <c r="P69" t="inlineStr">
         <is>
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/298?f=html</t>
+        </is>
+      </c>
+      <c r="Q69" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
     </row>
@@ -16024,7 +16403,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Denied</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -16061,6 +16440,11 @@
       <c r="P70" t="inlineStr">
         <is>
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/299?f=html</t>
+        </is>
+      </c>
+      <c r="Q70" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
     </row>
@@ -16075,7 +16459,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Denied</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -16112,6 +16496,11 @@
       <c r="P71" t="inlineStr">
         <is>
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/300?f=html</t>
+        </is>
+      </c>
+      <c r="Q71" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
     </row>
@@ -16126,7 +16515,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Denied</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -16163,6 +16552,11 @@
       <c r="P72" t="inlineStr">
         <is>
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/301?f=html</t>
+        </is>
+      </c>
+      <c r="Q72" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
     </row>
@@ -16177,7 +16571,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Denied</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -16214,6 +16608,11 @@
       <c r="P73" t="inlineStr">
         <is>
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/302?f=html</t>
+        </is>
+      </c>
+      <c r="Q73" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
     </row>
@@ -16228,7 +16627,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Denied</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -16265,6 +16664,11 @@
       <c r="P74" t="inlineStr">
         <is>
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/303?f=html</t>
+        </is>
+      </c>
+      <c r="Q74" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
     </row>
@@ -16279,7 +16683,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Denied</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -16316,6 +16720,11 @@
       <c r="P75" t="inlineStr">
         <is>
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/304?f=html</t>
+        </is>
+      </c>
+      <c r="Q75" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
     </row>
@@ -16330,7 +16739,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Denied</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -16367,6 +16776,11 @@
       <c r="P76" t="inlineStr">
         <is>
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/305?f=html</t>
+        </is>
+      </c>
+      <c r="Q76" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
     </row>
@@ -16381,7 +16795,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Denied</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -16418,6 +16832,11 @@
       <c r="P77" t="inlineStr">
         <is>
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/306?f=html</t>
+        </is>
+      </c>
+      <c r="Q77" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
     </row>
@@ -16432,7 +16851,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Denied</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -16469,6 +16888,11 @@
       <c r="P78" t="inlineStr">
         <is>
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/307?f=html</t>
+        </is>
+      </c>
+      <c r="Q78" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
     </row>
@@ -16483,7 +16907,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Denied</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -16520,6 +16944,11 @@
       <c r="P79" t="inlineStr">
         <is>
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/308?f=html</t>
+        </is>
+      </c>
+      <c r="Q79" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
     </row>
@@ -16534,7 +16963,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Denied</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -16571,6 +17000,11 @@
       <c r="P80" t="inlineStr">
         <is>
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/309?f=html</t>
+        </is>
+      </c>
+      <c r="Q80" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
     </row>
@@ -16585,7 +17019,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Denied</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -16622,6 +17056,11 @@
       <c r="P81" t="inlineStr">
         <is>
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/310?f=html</t>
+        </is>
+      </c>
+      <c r="Q81" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
     </row>
@@ -16636,7 +17075,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Denied</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -16673,6 +17112,11 @@
       <c r="P82" t="inlineStr">
         <is>
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/311?f=html</t>
+        </is>
+      </c>
+      <c r="Q82" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
     </row>
@@ -16687,7 +17131,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Denied</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -16724,6 +17168,11 @@
       <c r="P83" t="inlineStr">
         <is>
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/312?f=html</t>
+        </is>
+      </c>
+      <c r="Q83" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
     </row>
@@ -16738,7 +17187,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Denied</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -16775,6 +17224,11 @@
       <c r="P84" t="inlineStr">
         <is>
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/313?f=html</t>
+        </is>
+      </c>
+      <c r="Q84" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
     </row>
@@ -16851,6 +17305,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/83?f=html</t>
         </is>
       </c>
+      <c r="Q85" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -16925,6 +17384,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/87?f=html</t>
         </is>
       </c>
+      <c r="Q86" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -16999,6 +17463,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/84?f=html</t>
         </is>
       </c>
+      <c r="Q87" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -17065,6 +17534,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/86?f=html</t>
         </is>
       </c>
+      <c r="Q88" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -17126,6 +17600,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/85?f=html</t>
         </is>
       </c>
+      <c r="Q89" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -17187,6 +17666,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/678?f=html</t>
         </is>
       </c>
+      <c r="Q90" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -17243,6 +17727,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/127?f=html</t>
         </is>
       </c>
+      <c r="Q91" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -17299,6 +17788,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/126?f=html</t>
         </is>
       </c>
+      <c r="Q92" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -17355,6 +17849,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/124?f=html</t>
         </is>
       </c>
+      <c r="Q93" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -17411,6 +17910,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/122?f=html</t>
         </is>
       </c>
+      <c r="Q94" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -17467,6 +17971,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/125?f=html</t>
         </is>
       </c>
+      <c r="Q95" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -17523,6 +18032,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/123?f=html</t>
         </is>
       </c>
+      <c r="Q96" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -17579,6 +18093,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/121?f=html</t>
         </is>
       </c>
+      <c r="Q97" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -17635,6 +18154,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/128?f=html</t>
         </is>
       </c>
+      <c r="Q98" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -17647,7 +18171,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Denied</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -17684,6 +18208,11 @@
       <c r="P99" t="inlineStr">
         <is>
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/277?f=html</t>
+        </is>
+      </c>
+      <c r="Q99" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
     </row>
@@ -17698,7 +18227,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Denied</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -17735,6 +18264,11 @@
       <c r="P100" t="inlineStr">
         <is>
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/278?f=html</t>
+        </is>
+      </c>
+      <c r="Q100" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
     </row>
@@ -17749,7 +18283,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Denied</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -17786,6 +18320,11 @@
       <c r="P101" t="inlineStr">
         <is>
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/279?f=html</t>
+        </is>
+      </c>
+      <c r="Q101" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
     </row>
@@ -17800,7 +18339,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Denied</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -17837,6 +18376,11 @@
       <c r="P102" t="inlineStr">
         <is>
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/280?f=html</t>
+        </is>
+      </c>
+      <c r="Q102" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
     </row>
@@ -17851,7 +18395,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Denied</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -17888,6 +18432,11 @@
       <c r="P103" t="inlineStr">
         <is>
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/281?f=html</t>
+        </is>
+      </c>
+      <c r="Q103" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
     </row>
@@ -17902,7 +18451,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Denied</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -17939,6 +18488,11 @@
       <c r="P104" t="inlineStr">
         <is>
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/290?f=html</t>
+        </is>
+      </c>
+      <c r="Q104" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
     </row>
@@ -17953,7 +18507,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Denied</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -17990,6 +18544,11 @@
       <c r="P105" t="inlineStr">
         <is>
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/291?f=html</t>
+        </is>
+      </c>
+      <c r="Q105" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
     </row>
@@ -18004,7 +18563,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Denied</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -18041,6 +18600,11 @@
       <c r="P106" t="inlineStr">
         <is>
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/292?f=html</t>
+        </is>
+      </c>
+      <c r="Q106" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
     </row>
@@ -18055,7 +18619,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Denied</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -18092,6 +18656,11 @@
       <c r="P107" t="inlineStr">
         <is>
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/293?f=html</t>
+        </is>
+      </c>
+      <c r="Q107" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
     </row>
@@ -18106,7 +18675,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Denied</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -18143,6 +18712,11 @@
       <c r="P108" t="inlineStr">
         <is>
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/294?f=html</t>
+        </is>
+      </c>
+      <c r="Q108" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
     </row>
@@ -18157,7 +18731,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Denied</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -18194,6 +18768,11 @@
       <c r="P109" t="inlineStr">
         <is>
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/295?f=html</t>
+        </is>
+      </c>
+      <c r="Q109" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
     </row>
@@ -18208,7 +18787,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Denied</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -18245,6 +18824,11 @@
       <c r="P110" t="inlineStr">
         <is>
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/296?f=html</t>
+        </is>
+      </c>
+      <c r="Q110" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
     </row>
@@ -18259,7 +18843,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Denied</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -18296,6 +18880,11 @@
       <c r="P111" t="inlineStr">
         <is>
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/282?f=html</t>
+        </is>
+      </c>
+      <c r="Q111" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
     </row>
@@ -18310,7 +18899,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Denied</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -18347,6 +18936,11 @@
       <c r="P112" t="inlineStr">
         <is>
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/283?f=html</t>
+        </is>
+      </c>
+      <c r="Q112" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
     </row>
@@ -18361,7 +18955,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Denied</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -18398,6 +18992,11 @@
       <c r="P113" t="inlineStr">
         <is>
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/284?f=html</t>
+        </is>
+      </c>
+      <c r="Q113" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
     </row>
@@ -18412,7 +19011,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Denied</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -18449,6 +19048,11 @@
       <c r="P114" t="inlineStr">
         <is>
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/285?f=html</t>
+        </is>
+      </c>
+      <c r="Q114" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
     </row>
@@ -18463,7 +19067,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Denied</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -18500,6 +19104,11 @@
       <c r="P115" t="inlineStr">
         <is>
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/286?f=html</t>
+        </is>
+      </c>
+      <c r="Q115" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
     </row>
@@ -18514,7 +19123,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Denied</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -18551,6 +19160,11 @@
       <c r="P116" t="inlineStr">
         <is>
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/287?f=html</t>
+        </is>
+      </c>
+      <c r="Q116" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
     </row>
@@ -18565,7 +19179,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Denied</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -18602,6 +19216,11 @@
       <c r="P117" t="inlineStr">
         <is>
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/288?f=html</t>
+        </is>
+      </c>
+      <c r="Q117" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
     </row>
@@ -18616,7 +19235,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Denied</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -18653,6 +19272,11 @@
       <c r="P118" t="inlineStr">
         <is>
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/289?f=html</t>
+        </is>
+      </c>
+      <c r="Q118" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
     </row>
@@ -18721,6 +19345,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/59?f=html</t>
         </is>
       </c>
+      <c r="Q119" t="inlineStr">
+        <is>
+          <t>Under Construction</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -18790,6 +19419,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/58?f=html</t>
         </is>
       </c>
+      <c r="Q120" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -18864,6 +19498,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/96?f=html</t>
         </is>
       </c>
+      <c r="Q121" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -18925,6 +19564,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/243?f=html</t>
         </is>
       </c>
+      <c r="Q122" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -18999,6 +19643,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/154?f=html</t>
         </is>
       </c>
+      <c r="Q123" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -19065,6 +19714,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/272?f=html</t>
         </is>
       </c>
+      <c r="Q124" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -19129,6 +19783,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/215?f=html</t>
         </is>
       </c>
+      <c r="Q125" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -19185,6 +19844,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/143?f=html</t>
         </is>
       </c>
+      <c r="Q126" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="n">
@@ -19241,6 +19905,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/144?f=html</t>
         </is>
       </c>
+      <c r="Q127" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -19307,6 +19976,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/114?f=html</t>
         </is>
       </c>
+      <c r="Q128" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="n">
@@ -19373,6 +20047,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/78?f=html</t>
         </is>
       </c>
+      <c r="Q129" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -19429,6 +20108,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/140?f=html</t>
         </is>
       </c>
+      <c r="Q130" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -19485,6 +20169,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/155?f=html</t>
         </is>
       </c>
+      <c r="Q131" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -19541,6 +20230,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/156?f=html</t>
         </is>
       </c>
+      <c r="Q132" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -19597,6 +20291,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/157?f=html</t>
         </is>
       </c>
+      <c r="Q133" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -19653,6 +20352,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/158?f=html</t>
         </is>
       </c>
+      <c r="Q134" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -19727,6 +20431,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/32?f=html</t>
         </is>
       </c>
+      <c r="Q135" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -19798,6 +20507,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/30?f=html</t>
         </is>
       </c>
+      <c r="Q136" t="inlineStr">
+        <is>
+          <t>Under Construction</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -19864,6 +20578,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/31?f=html</t>
         </is>
       </c>
+      <c r="Q137" t="inlineStr">
+        <is>
+          <t>Under Construction</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -19925,6 +20644,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/216?f=html</t>
         </is>
       </c>
+      <c r="Q138" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -19986,6 +20710,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/220?f=html</t>
         </is>
       </c>
+      <c r="Q139" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -20047,6 +20776,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/204?f=html</t>
         </is>
       </c>
+      <c r="Q140" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -20103,6 +20837,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/163?f=html</t>
         </is>
       </c>
+      <c r="Q141" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -20159,6 +20898,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/172?f=html</t>
         </is>
       </c>
+      <c r="Q142" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="n">
@@ -20215,6 +20959,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/164?f=html</t>
         </is>
       </c>
+      <c r="Q143" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -20271,6 +21020,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/169?f=html</t>
         </is>
       </c>
+      <c r="Q144" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="n">
@@ -20327,6 +21081,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/168?f=html</t>
         </is>
       </c>
+      <c r="Q145" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -20383,6 +21142,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/167?f=html</t>
         </is>
       </c>
+      <c r="Q146" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="n">
@@ -20439,6 +21203,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/166?f=html</t>
         </is>
       </c>
+      <c r="Q147" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="n">
@@ -20495,6 +21264,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/165?f=html</t>
         </is>
       </c>
+      <c r="Q148" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="n">
@@ -20551,6 +21325,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/170?f=html</t>
         </is>
       </c>
+      <c r="Q149" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="n">
@@ -20607,6 +21386,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/171?f=html</t>
         </is>
       </c>
+      <c r="Q150" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="n">
@@ -20663,6 +21447,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/129?f=html</t>
         </is>
       </c>
+      <c r="Q151" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="n">
@@ -20732,6 +21521,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/1?f=html</t>
         </is>
       </c>
+      <c r="Q152" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="n">
@@ -20801,6 +21595,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/88?f=html</t>
         </is>
       </c>
+      <c r="Q153" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="n">
@@ -20870,6 +21669,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/2?f=html</t>
         </is>
       </c>
+      <c r="Q154" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="n">
@@ -20939,6 +21743,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/3?f=html</t>
         </is>
       </c>
+      <c r="Q155" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="n">
@@ -21008,6 +21817,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/4?f=html</t>
         </is>
       </c>
+      <c r="Q156" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="n">
@@ -21077,6 +21891,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/5?f=html</t>
         </is>
       </c>
+      <c r="Q157" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="n">
@@ -21146,6 +21965,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/6?f=html</t>
         </is>
       </c>
+      <c r="Q158" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="n">
@@ -21215,6 +22039,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/7?f=html</t>
         </is>
       </c>
+      <c r="Q159" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="n">
@@ -21284,6 +22113,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/8?f=html</t>
         </is>
       </c>
+      <c r="Q160" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="n">
@@ -21343,6 +22177,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/64?f=html</t>
         </is>
       </c>
+      <c r="Q161" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="n">
@@ -21402,6 +22241,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/66?f=html</t>
         </is>
       </c>
+      <c r="Q162" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="n">
@@ -21461,6 +22305,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/65?f=html</t>
         </is>
       </c>
+      <c r="Q163" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="n">
@@ -21522,6 +22371,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/223?f=html</t>
         </is>
       </c>
+      <c r="Q164" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="n">
@@ -21583,6 +22437,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/57?f=html</t>
         </is>
       </c>
+      <c r="Q165" t="inlineStr">
+        <is>
+          <t>Under Construction</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="n">
@@ -21649,6 +22508,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/240?f=html</t>
         </is>
       </c>
+      <c r="Q166" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="n">
@@ -21700,6 +22564,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/241?f=html</t>
         </is>
       </c>
+      <c r="Q167" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="n">
@@ -21761,6 +22630,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/271?f=html</t>
         </is>
       </c>
+      <c r="Q168" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="n">
@@ -21822,6 +22696,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/221?f=html</t>
         </is>
       </c>
+      <c r="Q169" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="n">
@@ -21883,6 +22762,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/222?f=html</t>
         </is>
       </c>
+      <c r="Q170" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="n">
@@ -21944,6 +22828,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/276?f=html</t>
         </is>
       </c>
+      <c r="Q171" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="n">
@@ -22005,6 +22894,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/275?f=html</t>
         </is>
       </c>
+      <c r="Q172" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="n">
@@ -22066,6 +22960,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/273?f=html</t>
         </is>
       </c>
+      <c r="Q173" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="n">
@@ -22127,6 +23026,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/274?f=html</t>
         </is>
       </c>
+      <c r="Q174" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="n">
@@ -22188,6 +23092,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/73?f=html</t>
         </is>
       </c>
+      <c r="Q175" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="n">
@@ -22247,6 +23156,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/74?f=html</t>
         </is>
       </c>
+      <c r="Q176" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="n">
@@ -22308,6 +23222,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/89?f=html</t>
         </is>
       </c>
+      <c r="Q177" t="inlineStr">
+        <is>
+          <t>Under Construction</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="n">
@@ -22372,6 +23291,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/90?f=html</t>
         </is>
       </c>
+      <c r="Q178" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="n">
@@ -22436,6 +23360,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/91?f=html</t>
         </is>
       </c>
+      <c r="Q179" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="n">
@@ -22500,6 +23429,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/92?f=html</t>
         </is>
       </c>
+      <c r="Q180" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="n">
@@ -22561,6 +23495,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/101?f=html</t>
         </is>
       </c>
+      <c r="Q181" t="inlineStr">
+        <is>
+          <t>Under Construction</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="n">
@@ -22622,6 +23561,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/104?f=html</t>
         </is>
       </c>
+      <c r="Q182" t="inlineStr">
+        <is>
+          <t>Under Construction</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="n">
@@ -22683,6 +23627,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/102?f=html</t>
         </is>
       </c>
+      <c r="Q183" t="inlineStr">
+        <is>
+          <t>Under Construction</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="n">
@@ -22739,6 +23688,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/103?f=html</t>
         </is>
       </c>
+      <c r="Q184" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="n">
@@ -22795,6 +23749,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/68?f=html</t>
         </is>
       </c>
+      <c r="Q185" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="n">
@@ -22851,6 +23810,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/71?f=html</t>
         </is>
       </c>
+      <c r="Q186" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="n">
@@ -22907,6 +23871,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/72?f=html</t>
         </is>
       </c>
+      <c r="Q187" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="n">
@@ -22963,6 +23932,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/226?f=html</t>
         </is>
       </c>
+      <c r="Q188" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="n">
@@ -23024,6 +23998,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/677?f=html</t>
         </is>
       </c>
+      <c r="Q189" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="n">
@@ -23090,6 +24069,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/77?f=html</t>
         </is>
       </c>
+      <c r="Q190" t="inlineStr">
+        <is>
+          <t>Under Construction</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="n">
@@ -23156,6 +24140,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/111?f=html</t>
         </is>
       </c>
+      <c r="Q191" t="inlineStr">
+        <is>
+          <t>Under Construction</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="n">
@@ -23222,6 +24211,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/112?f=html</t>
         </is>
       </c>
+      <c r="Q192" t="inlineStr">
+        <is>
+          <t>Under Construction</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="n">
@@ -23288,6 +24282,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/113?f=html</t>
         </is>
       </c>
+      <c r="Q193" t="inlineStr">
+        <is>
+          <t>Under Construction</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="n">
@@ -23349,6 +24348,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/210?f=html</t>
         </is>
       </c>
+      <c r="Q194" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="n">
@@ -23410,6 +24414,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/208?f=html</t>
         </is>
       </c>
+      <c r="Q195" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="n">
@@ -23471,6 +24480,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/209?f=html</t>
         </is>
       </c>
+      <c r="Q196" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="n">
@@ -23532,6 +24546,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/679?f=html</t>
         </is>
       </c>
+      <c r="Q197" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="n">
@@ -23593,6 +24612,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/206?f=html</t>
         </is>
       </c>
+      <c r="Q198" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="n">
@@ -23654,6 +24678,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/207?f=html</t>
         </is>
       </c>
+      <c r="Q199" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="n">
@@ -23715,6 +24744,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/160?f=html</t>
         </is>
       </c>
+      <c r="Q200" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="n">
@@ -23776,6 +24810,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/161?f=html</t>
         </is>
       </c>
+      <c r="Q201" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="n">
@@ -23850,6 +24889,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/23?f=html</t>
         </is>
       </c>
+      <c r="Q202" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="n">
@@ -23924,6 +24968,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/25?f=html</t>
         </is>
       </c>
+      <c r="Q203" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="n">
@@ -23998,6 +25047,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/24?f=html</t>
         </is>
       </c>
+      <c r="Q204" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="n">
@@ -24064,6 +25118,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/26?f=html</t>
         </is>
       </c>
+      <c r="Q205" t="inlineStr">
+        <is>
+          <t>Under Construction</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="n">
@@ -24133,6 +25192,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/22?f=html</t>
         </is>
       </c>
+      <c r="Q206" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="n">
@@ -24199,6 +25263,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/21?f=html</t>
         </is>
       </c>
+      <c r="Q207" t="inlineStr">
+        <is>
+          <t>Under Construction</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="n">
@@ -24260,6 +25329,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/231?f=html</t>
         </is>
       </c>
+      <c r="Q208" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="n">
@@ -24321,6 +25395,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/232?f=html</t>
         </is>
       </c>
+      <c r="Q209" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="n">
@@ -24382,6 +25461,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/239?f=html</t>
         </is>
       </c>
+      <c r="Q210" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="n">
@@ -24443,6 +25527,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/238?f=html</t>
         </is>
       </c>
+      <c r="Q211" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="n">
@@ -24504,6 +25593,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/237?f=html</t>
         </is>
       </c>
+      <c r="Q212" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="n">
@@ -24565,6 +25659,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/236?f=html</t>
         </is>
       </c>
+      <c r="Q213" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="n">
@@ -24626,6 +25725,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/235?f=html</t>
         </is>
       </c>
+      <c r="Q214" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="n">
@@ -24687,6 +25791,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/225?f=html</t>
         </is>
       </c>
+      <c r="Q215" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" t="n">
@@ -24748,6 +25857,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/224?f=html</t>
         </is>
       </c>
+      <c r="Q216" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" t="n">
@@ -24809,6 +25923,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/218?f=html</t>
         </is>
       </c>
+      <c r="Q217" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="n">
@@ -24870,6 +25989,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/217?f=html</t>
         </is>
       </c>
+      <c r="Q218" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" t="n">
@@ -24931,6 +26055,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/219?f=html</t>
         </is>
       </c>
+      <c r="Q219" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="n">
@@ -24992,6 +26121,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/229?f=html</t>
         </is>
       </c>
+      <c r="Q220" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="221">
       <c r="A221" t="n">
@@ -25053,6 +26187,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/230?f=html</t>
         </is>
       </c>
+      <c r="Q221" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" t="n">
@@ -25122,6 +26261,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/11?f=html</t>
         </is>
       </c>
+      <c r="Q222" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="n">
@@ -25183,6 +26327,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/12?f=html</t>
         </is>
       </c>
+      <c r="Q223" t="inlineStr">
+        <is>
+          <t>Under Construction</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" t="n">
@@ -25244,6 +26393,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/262?f=html</t>
         </is>
       </c>
+      <c r="Q224" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" t="n">
@@ -25305,6 +26459,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/264?f=html</t>
         </is>
       </c>
+      <c r="Q225" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="n">
@@ -25366,6 +26525,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/263?f=html</t>
         </is>
       </c>
+      <c r="Q226" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" t="n">
@@ -25435,6 +26599,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/37?f=html</t>
         </is>
       </c>
+      <c r="Q227" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" t="n">
@@ -25504,6 +26673,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/38?f=html</t>
         </is>
       </c>
+      <c r="Q228" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="n">
@@ -25573,6 +26747,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/39?f=html</t>
         </is>
       </c>
+      <c r="Q229" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="n">
@@ -25642,6 +26821,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/40?f=html</t>
         </is>
       </c>
+      <c r="Q230" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" t="n">
@@ -25711,6 +26895,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/42?f=html</t>
         </is>
       </c>
+      <c r="Q231" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" t="n">
@@ -25772,6 +26961,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/45?f=html</t>
         </is>
       </c>
+      <c r="Q232" t="inlineStr">
+        <is>
+          <t>Under Construction</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="n">
@@ -25838,6 +27032,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/41?f=html</t>
         </is>
       </c>
+      <c r="Q233" t="inlineStr">
+        <is>
+          <t>Under Construction</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" t="n">
@@ -25904,6 +27103,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/43?f=html</t>
         </is>
       </c>
+      <c r="Q234" t="inlineStr">
+        <is>
+          <t>Under Construction</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" t="n">
@@ -25970,6 +27174,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/44?f=html</t>
         </is>
       </c>
+      <c r="Q235" t="inlineStr">
+        <is>
+          <t>Under Construction</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" t="n">
@@ -26036,6 +27245,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/63?f=html</t>
         </is>
       </c>
+      <c r="Q236" t="inlineStr">
+        <is>
+          <t>Under Construction</t>
+        </is>
+      </c>
     </row>
     <row r="237">
       <c r="A237" t="n">
@@ -26097,6 +27311,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/33?f=html</t>
         </is>
       </c>
+      <c r="Q237" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="238">
       <c r="A238" t="n">
@@ -26153,6 +27372,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/245?f=html</t>
         </is>
       </c>
+      <c r="Q238" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="239">
       <c r="A239" t="n">
@@ -26214,6 +27438,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/680?f=html</t>
         </is>
       </c>
+      <c r="Q239" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="240">
       <c r="A240" t="n">
@@ -26288,6 +27517,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/29?f=html</t>
         </is>
       </c>
+      <c r="Q240" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="241">
       <c r="A241" t="n">
@@ -26349,6 +27583,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/116?f=html</t>
         </is>
       </c>
+      <c r="Q241" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="242">
       <c r="A242" t="n">
@@ -26410,6 +27649,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/118?f=html</t>
         </is>
       </c>
+      <c r="Q242" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="243">
       <c r="A243" t="n">
@@ -26479,6 +27723,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/153?f=html</t>
         </is>
       </c>
+      <c r="Q243" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="244">
       <c r="A244" t="n">
@@ -26535,6 +27784,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/110?f=html</t>
         </is>
       </c>
+      <c r="Q244" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
     </row>
     <row r="245">
       <c r="A245" t="n">
@@ -26609,6 +27863,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/93?f=html</t>
         </is>
       </c>
+      <c r="Q245" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="246">
       <c r="A246" t="n">
@@ -26683,6 +27942,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/94?f=html</t>
         </is>
       </c>
+      <c r="Q246" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="247">
       <c r="A247" t="n">
@@ -26757,6 +28021,11 @@
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/95?f=html</t>
         </is>
       </c>
+      <c r="Q247" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="248">
       <c r="A248" t="n">
@@ -26821,6 +28090,11 @@
       <c r="P248" t="inlineStr">
         <is>
           <t>https://gisweb.pwcva.gov/arcgis/rest/services/Planning/Build_Out_Analysis/MapServer/9/258?f=html</t>
+        </is>
+      </c>
+      <c r="Q248" t="inlineStr">
+        <is>
+          <t>Planned</t>
         </is>
       </c>
     </row>

</xml_diff>